<commit_message>
chore: synchronize timetable data
</commit_message>
<xml_diff>
--- a/raw_data/1-62.xlsx
+++ b/raw_data/1-62.xlsx
@@ -142,6 +142,40 @@
       <left style="thin">
         <color rgb="00000000"/>
       </left>
+      <right>
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal>
+        <color rgb="00000000"/>
+      </diagonal>
+    </border>
+    <border>
+      <left>
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal>
+        <color rgb="00000000"/>
+      </diagonal>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
       <right style="thin">
         <color rgb="00000000"/>
       </right>
@@ -166,40 +200,6 @@
         <color rgb="00000000"/>
       </top>
       <bottom>
-        <color rgb="00000000"/>
-      </bottom>
-      <diagonal>
-        <color rgb="00000000"/>
-      </diagonal>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right>
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
-      <diagonal>
-        <color rgb="00000000"/>
-      </diagonal>
-    </border>
-    <border>
-      <left>
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
         <color rgb="00000000"/>
       </bottom>
       <diagonal>
@@ -2723,8 +2723,12 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="19" t="n"/>
-      <c r="B38" s="12" t="inlineStr"/>
-      <c r="C38" s="12" t="inlineStr"/>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>PC1(EC112)-EDC/SL,M,RRP</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n"/>
       <c r="D38" s="12" t="inlineStr"/>
       <c r="E38" s="19" t="n"/>
       <c r="F38" s="10" t="inlineStr">
@@ -3667,7 +3671,7 @@
       <c r="C59" s="13" t="inlineStr"/>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>TA8(EC111)-/JG</t>
+          <t>TA8(EC111)-F10/JG</t>
         </is>
       </c>
       <c r="E59" s="11" t="n"/>
@@ -4528,11 +4532,7 @@
           <t>LA15,A16(PH111)-FF2/DIN</t>
         </is>
       </c>
-      <c r="G81" s="10" t="inlineStr">
-        <is>
-          <t>LA15,A16(EC111)-FF2/RRJ</t>
-        </is>
-      </c>
+      <c r="G81" s="12" t="inlineStr"/>
       <c r="H81" s="10" t="inlineStr">
         <is>
           <t>LB1,B2(CI111)-FF2/TNV</t>
@@ -4901,7 +4901,11 @@
       <c r="A89" s="11" t="n"/>
       <c r="B89" s="10" t="inlineStr"/>
       <c r="C89" s="12" t="inlineStr"/>
-      <c r="D89" s="12" t="inlineStr"/>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>LA15,A16(EC111)-CR301/RRJ</t>
+        </is>
+      </c>
       <c r="E89" s="11" t="n"/>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5807,12 +5811,8 @@
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="11" t="n"/>
-      <c r="B111" s="10" t="inlineStr">
-        <is>
-          <t>PC1(EC112)-EDC/SL,M,RRP</t>
-        </is>
-      </c>
-      <c r="C111" s="4" t="n"/>
+      <c r="B111" s="12" t="inlineStr"/>
+      <c r="C111" s="12" t="inlineStr"/>
       <c r="D111" s="10" t="inlineStr"/>
       <c r="E111" s="11" t="n"/>
       <c r="F111" s="16" t="inlineStr">
@@ -6835,11 +6835,7 @@
       </c>
       <c r="D134" s="12" t="inlineStr"/>
       <c r="E134" s="11" t="n"/>
-      <c r="F134" s="10" t="inlineStr">
-        <is>
-          <t>TB4(EC111)-F7/RHA</t>
-        </is>
-      </c>
+      <c r="F134" s="12" t="inlineStr"/>
       <c r="G134" s="10" t="inlineStr">
         <is>
           <t>TB13(PH111)-F7/SND</t>
@@ -8020,7 +8016,11 @@
           <t>LB13,B14(HS112)-G7/KNP</t>
         </is>
       </c>
-      <c r="G162" s="12" t="inlineStr"/>
+      <c r="G162" s="10" t="inlineStr">
+        <is>
+          <t>TB4(EC111)-TS16/RHA</t>
+        </is>
+      </c>
       <c r="H162" s="13" t="inlineStr">
         <is>
           <t>LH1,H2(EC111)-G8/ATA</t>
@@ -32892,39 +32892,40 @@
     <mergeCell ref="F29:G29"/>
     <mergeCell ref="H181:I181"/>
     <mergeCell ref="F68:G68"/>
+    <mergeCell ref="F103:G103"/>
     <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F103:G103"/>
     <mergeCell ref="F174:G174"/>
+    <mergeCell ref="F108:G108"/>
     <mergeCell ref="C107:D107"/>
-    <mergeCell ref="F108:G108"/>
     <mergeCell ref="A190:A223"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B215:C215"/>
+    <mergeCell ref="C64:D64"/>
     <mergeCell ref="F143:G143"/>
-    <mergeCell ref="C64:D64"/>
     <mergeCell ref="H180:I180"/>
     <mergeCell ref="H143:I143"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="F115:H115"/>
+    <mergeCell ref="F173:G173"/>
     <mergeCell ref="B228:I228"/>
+    <mergeCell ref="C63:D63"/>
     <mergeCell ref="D213:E213"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="C177:D177"/>
     <mergeCell ref="F142:G142"/>
-    <mergeCell ref="C177:D177"/>
-    <mergeCell ref="C63:D63"/>
     <mergeCell ref="H142:I142"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="F173:G173"/>
     <mergeCell ref="C173:D173"/>
     <mergeCell ref="F152:H152"/>
     <mergeCell ref="H108:I108"/>
+    <mergeCell ref="C105:D105"/>
     <mergeCell ref="F144:G144"/>
-    <mergeCell ref="C105:D105"/>
     <mergeCell ref="B69:C69"/>
     <mergeCell ref="H144:I144"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B178:C178"/>
+    <mergeCell ref="A79:A116"/>
     <mergeCell ref="C138:D138"/>
-    <mergeCell ref="A79:A116"/>
-    <mergeCell ref="B178:C178"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="B211:C211"/>
     <mergeCell ref="H65:I65"/>
@@ -32934,34 +32935,34 @@
     <mergeCell ref="E79:E116"/>
     <mergeCell ref="G36:I36"/>
     <mergeCell ref="H139:I139"/>
+    <mergeCell ref="H62:I62"/>
     <mergeCell ref="D237:I237"/>
-    <mergeCell ref="H62:I62"/>
     <mergeCell ref="A225:I225"/>
     <mergeCell ref="F107:G107"/>
+    <mergeCell ref="H23:I23"/>
     <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B219:D219"/>
     <mergeCell ref="H107:I107"/>
-    <mergeCell ref="B219:D219"/>
-    <mergeCell ref="H23:I23"/>
     <mergeCell ref="B212:C212"/>
     <mergeCell ref="F175:G175"/>
+    <mergeCell ref="A227:I227"/>
     <mergeCell ref="F113:H113"/>
-    <mergeCell ref="A227:I227"/>
     <mergeCell ref="B209:C209"/>
     <mergeCell ref="C175:D175"/>
     <mergeCell ref="F114:H114"/>
     <mergeCell ref="F63:G63"/>
+    <mergeCell ref="F34:G34"/>
     <mergeCell ref="B232:I232"/>
-    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H63:I63"/>
     <mergeCell ref="F146:G146"/>
-    <mergeCell ref="H63:I63"/>
+    <mergeCell ref="B66:C66"/>
     <mergeCell ref="H146:I146"/>
-    <mergeCell ref="B66:C66"/>
     <mergeCell ref="A155:A188"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="H102:I102"/>
     <mergeCell ref="H68:I68"/>
+    <mergeCell ref="H34:I34"/>
     <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H34:I34"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F138:G138"/>
     <mergeCell ref="A234:I234"/>
@@ -32972,23 +32973,23 @@
     <mergeCell ref="B179:C179"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="F66:G66"/>
+    <mergeCell ref="H69:I69"/>
     <mergeCell ref="H182:I182"/>
+    <mergeCell ref="B36:D36"/>
     <mergeCell ref="F109:G109"/>
-    <mergeCell ref="F151:H151"/>
-    <mergeCell ref="C139:D139"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="H109:I109"/>
     <mergeCell ref="F62:G62"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="H69:I69"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="H109:I109"/>
+    <mergeCell ref="C139:D139"/>
+    <mergeCell ref="F151:H151"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B75:D75"/>
     <mergeCell ref="F111:G111"/>
     <mergeCell ref="F116:H116"/>
-    <mergeCell ref="B75:D75"/>
     <mergeCell ref="H111:I111"/>
+    <mergeCell ref="H28:I28"/>
     <mergeCell ref="F61:G61"/>
     <mergeCell ref="B150:D150"/>
     <mergeCell ref="C174:D174"/>
@@ -33002,153 +33003,152 @@
     <mergeCell ref="E118:E153"/>
     <mergeCell ref="F64:G64"/>
     <mergeCell ref="H106:I106"/>
+    <mergeCell ref="F178:G178"/>
     <mergeCell ref="F147:G147"/>
-    <mergeCell ref="F178:G178"/>
+    <mergeCell ref="B185:C185"/>
     <mergeCell ref="B72:C72"/>
     <mergeCell ref="H147:I147"/>
-    <mergeCell ref="B185:C185"/>
     <mergeCell ref="B181:D181"/>
+    <mergeCell ref="C141:D141"/>
     <mergeCell ref="D208:E208"/>
     <mergeCell ref="F137:G137"/>
-    <mergeCell ref="C141:D141"/>
     <mergeCell ref="F153:H153"/>
     <mergeCell ref="H137:I137"/>
     <mergeCell ref="H31:I31"/>
-    <mergeCell ref="G211:H211"/>
+    <mergeCell ref="B71:C71"/>
     <mergeCell ref="H58:I58"/>
-    <mergeCell ref="B71:C71"/>
     <mergeCell ref="F185:H185"/>
     <mergeCell ref="B214:C214"/>
     <mergeCell ref="F38:H38"/>
     <mergeCell ref="B210:C210"/>
     <mergeCell ref="C143:D143"/>
+    <mergeCell ref="C100:D100"/>
     <mergeCell ref="F139:G139"/>
-    <mergeCell ref="C100:D100"/>
+    <mergeCell ref="F71:H71"/>
+    <mergeCell ref="D235:I235"/>
+    <mergeCell ref="H173:I173"/>
     <mergeCell ref="H60:I60"/>
-    <mergeCell ref="H173:I173"/>
-    <mergeCell ref="D235:I235"/>
-    <mergeCell ref="F71:H71"/>
     <mergeCell ref="E3:E38"/>
     <mergeCell ref="B183:D183"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="C142:D142"/>
-    <mergeCell ref="F110:G110"/>
+    <mergeCell ref="F101:G101"/>
     <mergeCell ref="C176:D176"/>
-    <mergeCell ref="B148:C148"/>
-    <mergeCell ref="F181:G181"/>
-    <mergeCell ref="F186:H186"/>
     <mergeCell ref="F37:H37"/>
     <mergeCell ref="H110:I110"/>
-    <mergeCell ref="F101:G101"/>
+    <mergeCell ref="F186:H186"/>
+    <mergeCell ref="F181:G181"/>
+    <mergeCell ref="F110:G110"/>
+    <mergeCell ref="B148:C148"/>
     <mergeCell ref="A40:A77"/>
+    <mergeCell ref="F100:G100"/>
+    <mergeCell ref="C21:D21"/>
     <mergeCell ref="B114:D114"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F100:G100"/>
     <mergeCell ref="G150:I150"/>
     <mergeCell ref="F180:G180"/>
     <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B221:D221"/>
+    <mergeCell ref="B146:C146"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="H174:I174"/>
     <mergeCell ref="B230:I230"/>
     <mergeCell ref="D212:E212"/>
+    <mergeCell ref="B221:D221"/>
     <mergeCell ref="F141:G141"/>
+    <mergeCell ref="B108:C108"/>
     <mergeCell ref="A118:A153"/>
-    <mergeCell ref="H174:I174"/>
-    <mergeCell ref="B146:C146"/>
-    <mergeCell ref="B108:C108"/>
-    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="H66:I66"/>
+    <mergeCell ref="F179:G179"/>
     <mergeCell ref="B113:D113"/>
-    <mergeCell ref="H66:I66"/>
+    <mergeCell ref="F102:G102"/>
     <mergeCell ref="C23:D23"/>
-    <mergeCell ref="F102:G102"/>
     <mergeCell ref="C106:D106"/>
     <mergeCell ref="F187:H187"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B115:D115"/>
     <mergeCell ref="B149:D149"/>
+    <mergeCell ref="B216:C216"/>
     <mergeCell ref="G212:H212"/>
     <mergeCell ref="B220:D220"/>
-    <mergeCell ref="B216:C216"/>
     <mergeCell ref="A235:A237"/>
     <mergeCell ref="H141:I141"/>
     <mergeCell ref="C140:D140"/>
     <mergeCell ref="B77:D77"/>
     <mergeCell ref="H30:I30"/>
     <mergeCell ref="H175:I175"/>
+    <mergeCell ref="C101:D101"/>
     <mergeCell ref="B109:C109"/>
+    <mergeCell ref="H67:I67"/>
+    <mergeCell ref="F182:G182"/>
+    <mergeCell ref="B218:C218"/>
+    <mergeCell ref="C24:D24"/>
     <mergeCell ref="B151:D151"/>
-    <mergeCell ref="B218:C218"/>
-    <mergeCell ref="F182:G182"/>
-    <mergeCell ref="H67:I67"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C101:D101"/>
     <mergeCell ref="H103:I103"/>
+    <mergeCell ref="F112:G112"/>
     <mergeCell ref="H29:I29"/>
-    <mergeCell ref="F112:G112"/>
-    <mergeCell ref="F183:G183"/>
+    <mergeCell ref="C104:D104"/>
     <mergeCell ref="F65:G65"/>
     <mergeCell ref="F188:H188"/>
-    <mergeCell ref="C104:D104"/>
+    <mergeCell ref="F183:G183"/>
     <mergeCell ref="F70:H70"/>
     <mergeCell ref="B116:D116"/>
+    <mergeCell ref="C26:D26"/>
     <mergeCell ref="B182:D182"/>
-    <mergeCell ref="C26:D26"/>
     <mergeCell ref="H176:I176"/>
     <mergeCell ref="C222:E222"/>
+    <mergeCell ref="B112:D112"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="F72:H72"/>
+    <mergeCell ref="F190:H190"/>
+    <mergeCell ref="F24:G24"/>
     <mergeCell ref="F59:G59"/>
-    <mergeCell ref="F190:H190"/>
-    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="F177:G177"/>
     <mergeCell ref="H59:I59"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F72:H72"/>
-    <mergeCell ref="F177:G177"/>
-    <mergeCell ref="B112:D112"/>
+    <mergeCell ref="H64:I64"/>
+    <mergeCell ref="F104:G104"/>
+    <mergeCell ref="C103:D103"/>
+    <mergeCell ref="C25:D25"/>
     <mergeCell ref="H177:I177"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="H64:I64"/>
-    <mergeCell ref="C103:D103"/>
-    <mergeCell ref="F104:G104"/>
-    <mergeCell ref="B111:C111"/>
+    <mergeCell ref="C99:D99"/>
     <mergeCell ref="B145:C145"/>
-    <mergeCell ref="C99:D99"/>
     <mergeCell ref="G35:I35"/>
     <mergeCell ref="H178:I178"/>
     <mergeCell ref="B231:I231"/>
+    <mergeCell ref="F145:G145"/>
     <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F145:G145"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="D236:I236"/>
     <mergeCell ref="D210:E210"/>
     <mergeCell ref="F26:G26"/>
+    <mergeCell ref="D236:I236"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="F106:G106"/>
     <mergeCell ref="B73:C73"/>
     <mergeCell ref="B33:D33"/>
-    <mergeCell ref="F106:G106"/>
     <mergeCell ref="B147:C147"/>
+    <mergeCell ref="D209:E209"/>
     <mergeCell ref="A265:I265"/>
-    <mergeCell ref="D209:E209"/>
     <mergeCell ref="H138:I138"/>
     <mergeCell ref="H32:I32"/>
+    <mergeCell ref="F73:H73"/>
+    <mergeCell ref="F184:G184"/>
     <mergeCell ref="B153:D153"/>
-    <mergeCell ref="F184:G184"/>
-    <mergeCell ref="F73:H73"/>
     <mergeCell ref="B217:C217"/>
+    <mergeCell ref="D211:E211"/>
+    <mergeCell ref="F27:G27"/>
     <mergeCell ref="E155:E188"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="F140:G140"/>
-    <mergeCell ref="D211:E211"/>
-    <mergeCell ref="H140:I140"/>
-    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="B65:C65"/>
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="F67:G67"/>
-    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="F140:G140"/>
+    <mergeCell ref="H140:I140"/>
+    <mergeCell ref="F58:G58"/>
     <mergeCell ref="B68:C68"/>
     <mergeCell ref="H101:I101"/>
+    <mergeCell ref="B184:D184"/>
     <mergeCell ref="H24:I24"/>
-    <mergeCell ref="B184:D184"/>
     <mergeCell ref="F60:G60"/>
     <mergeCell ref="H33:I33"/>
     <mergeCell ref="A3:A38"/>
     <mergeCell ref="B110:C110"/>
-    <mergeCell ref="F179:G179"/>
+    <mergeCell ref="G211:H211"/>
     <mergeCell ref="C136:D136"/>
     <mergeCell ref="H179:I179"/>
     <mergeCell ref="E40:E77"/>

</xml_diff>